<commit_message>
#42 Main Baseboard Board order 10 PCS.
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v2.0/BOM/JLCPCB-BOM-Baseboard-v2.0.xlsx
+++ b/Design Files/Baseboard-v2.0/BOM/JLCPCB-BOM-Baseboard-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="284">
   <si>
     <t>Comment</t>
   </si>
@@ -859,6 +859,18 @@
   </si>
   <si>
     <t>C362352</t>
+  </si>
+  <si>
+    <t>C542993</t>
+  </si>
+  <si>
+    <t>C705793</t>
+  </si>
+  <si>
+    <t>C266196</t>
+  </si>
+  <si>
+    <t>C661296</t>
   </si>
 </sst>
 </file>
@@ -1891,7 +1903,9 @@
       <c r="C42" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D42" s="4"/>
+      <c r="D42" s="4" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
@@ -2099,7 +2113,9 @@
       <c r="C57" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="D57" s="4"/>
+      <c r="D57" s="4" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
@@ -2207,7 +2223,9 @@
       <c r="C65" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="4"/>
+      <c r="D65" s="4" t="s">
+        <v>282</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
@@ -2329,7 +2347,9 @@
       <c r="C74" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="D74" s="6"/>
+      <c r="D74" s="6" t="s">
+        <v>283</v>
+      </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">

</xml_diff>